<commit_message>
Add nine reviewed NEU, CQU and SYSU academic profiles (993 total)
</commit_message>
<xml_diff>
--- a/site/exports/cqu-mathematics-statistics.xlsx
+++ b/site/exports/cqu-mathematics-statistics.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -675,12 +675,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>数学与统计学院</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/index.htm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>个人页分离姓名、讲师及所在单位数学与统计学院字段拼接，非连续引文；所属单位是本人页声明，独立目录匹配与当前在岗未核实。；博士毕业月2020-06与实际授位日期分开；本科具体理学学士学位称谓保留，不将学习终点认作授位日。；纽约州立大学Albany分校联合培养及复旦大学博士后均为非学位经历，不造额外授位或导师。；两篇选定作品非完整书目；2024及to appear保持原状态，未外核或更新为当前出版状态。；仅必要留存职业摘录，非完整HTTP或整页存档；分离字段的连接已标明。作品原生URL经阅读器链接解析后查重，不声称此前已独立验证目录或浏览器点击。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -692,13 +746,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="29.4" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22.4" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -2065,8 +2119,329 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2014-09</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2020-06</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>原2014.9–2020.6重庆大学数学学习；简介明确2020年6月博士毕业并获博士学位。保留毕业月，不将其另填为授位月；分离字段拼接不是连续引文。</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/index.htm</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>理学学士学位</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2010-09</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2014-06</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>数学与应用数学</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>原2010.9–2014.6重庆大学数学与应用数学，具体资格列理学学士学位；保留学习区间，不把结束时间当授位日期。</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/index.htm</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_training</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>美国纽约州立大学Albany分校</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2017-09</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2019-09</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>原2017年9月至2019年9月在美国纽约州立大学Albany分校联合培养，非独立第二次学位授予；不补导师。</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/index.htm</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_training</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>复旦大学</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2020-07</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>原2020年7月至2023年8月在复旦大学从事博士后研究，博士后为非学位经历，不推为额外学位。</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/index.htm</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>机构工作</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>原明确博士后出站后在重庆大学数学与统计学院工作，未给独立入职日期；个人页另列讲师，不把博士后结束月当入职或讲师起任。</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/index.htm</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S21"/>
+  <autoFilter ref="A1:S26"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -2088,6 +2463,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2190,19 +2570,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
@@ -2269,8 +2649,100 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Generalized multiplicative Hilbert operators on Hilbert spaces of Dirichlet series</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文（官网书目）</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/lwcg/400688/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>原作者顺序：Xiangdi Fu、Kunyu Guo、Fugang Yan；Studia Mathematica，2024，to appear；保留来源待刊状态，不更新成已正式发表。仅官网书目，未核出版者或全文，不由合作者推导师。</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Coanalytic models for the Hardy type operators</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文（官网书目）</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/lwcg/400688/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>原作者顺序：Xiangdi Fu、Kunyu Guo、Fugang Yan；Science China Mathematics，2024，67(12):2771–2788。仅官网书目，未核出版者或全文，不由合作者推导师。</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L3"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2281,7 +2753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2700,8 +3172,74 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>cqu-yan-profile</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/index.htm</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>晏福刚</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>cqu-yan-works</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.cqu.edu.cn/yanfugang/zh_CN/lwcg/400688/list/index.htm</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>cqu</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>重庆大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
+  <autoFilter ref="A1:G13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -2713,6 +3251,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>